<commit_message>
Ready for Render deployment
</commit_message>
<xml_diff>
--- a/exports/invoice.xlsx
+++ b/exports/invoice.xlsx
@@ -428,16 +428,16 @@
   <dimension ref="A1:J2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="40" customWidth="1" min="1" max="1"/>
-    <col width="21" customWidth="1" min="2" max="2"/>
+    <col width="33" customWidth="1" min="1" max="1"/>
+    <col width="19" customWidth="1" min="2" max="2"/>
     <col width="17" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="13" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="6" max="6"/>
     <col width="16" customWidth="1" min="7" max="7"/>
     <col width="19" customWidth="1" min="8" max="8"/>
     <col width="13" customWidth="1" min="9" max="9"/>
-    <col width="33" customWidth="1" min="10" max="10"/>
+    <col width="24" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -495,48 +495,40 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Damson Technologies Private Limited</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>FAH8FJ2200735892</t>
-        </is>
-      </c>
+          <t>Lokmat Media Private Limited</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr">
         <is>
-          <t>AABCD3982G</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>06AABCD3982G1ZP</t>
-        </is>
-      </c>
+          <t>14-6-2025</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>49144.07</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>8845.93</t>
-        </is>
-      </c>
+          <t>36,590.00</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
-          <t>57990.00</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr"/>
+          <t>36,590.00</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Cheque</t>
+        </is>
+      </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>₹</t>
+          <t>INR</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>OD223726052458816000 (1).pdf</t>
+          <t>Ventures 031294.pdf</t>
         </is>
       </c>
     </row>

</xml_diff>